<commit_message>
Deploy: exported workbook shows its figures
</commit_message>
<xml_diff>
--- a/assets/assets/templates/personal-budget.xlsx
+++ b/assets/assets/templates/personal-budget.xlsx
@@ -12695,9 +12695,11 @@
       </c>
       <c r="D99" s="73">
         <f>(2360.13+2186.48+240)-2700</f>
+        <v>2086.6100000000006</v>
       </c>
       <c r="E99" s="10">
         <f>(917.76+7108.59)-(2700+2086.61)</f>
+        <v>3239.74</v>
       </c>
       <c r="F99" s="10"/>
       <c r="G99" s="10"/>
@@ -13044,11 +13046,13 @@
       </c>
       <c r="D135" s="79">
         <f>SUM(B115:B134)</f>
+        <v>710.21999999999991</v>
       </c>
       <c r="F135" s="51"/>
       <c r="G135" s="51"/>
       <c r="H135" s="51">
         <f>SUM(I115:I134)</f>
+        <v>30</v>
       </c>
     </row>
     <row r="159" spans="2:2" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>